<commit_message>
FIX on utility; REFACTOR on emition
</commit_message>
<xml_diff>
--- a/test/fixtures/business_tenant.xlsx
+++ b/test/fixtures/business_tenant.xlsx
@@ -33,7 +33,7 @@
     <t>regularTenantAmount</t>
   </si>
   <si>
-    <t>Gas</t>
+    <t>Cooling</t>
   </si>
   <si>
     <t>Site 456</t>
@@ -334,11 +334,11 @@
       <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1">
-        <v>200.0</v>
+      <c r="D2" s="3">
+        <v>2022.0</v>
       </c>
-      <c r="E2" s="1">
-        <v>200.0</v>
+      <c r="E2" s="3">
+        <v>2222.0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>